<commit_message>
build based on a7b7633
</commit_message>
<xml_diff>
--- a/dev/02_-_JULIA2_-_Scientific_programming_with_Julia/outdata.xlsx
+++ b/dev/02_-_JULIA2_-_Scientific_programming_with_Julia/outdata.xlsx
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="myData" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr fullCalcOnLoad="1" calcMode="auto"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
   <si>
     <t>Country</t>
   </si>
@@ -421,13 +421,13 @@
       <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="n">
         <v>2000</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>11.354</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>3381.0</v>
       </c>
     </row>
@@ -435,13 +435,13 @@
       <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="n">
         <v>2000</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>15.288</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>2254.28</v>
       </c>
     </row>
@@ -449,13 +449,13 @@
       <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4">
+      <c r="B4" t="n">
         <v>2000</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>8.36925</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>1058.71</v>
       </c>
     </row>
@@ -463,13 +463,13 @@
       <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="B5">
+      <c r="B5" t="n">
         <v>2000</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>28.163</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>3184.67</v>
       </c>
     </row>
@@ -477,13 +477,13 @@
       <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B6">
+      <c r="B6" t="n">
         <v>2020</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>11.419</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>3663.0</v>
       </c>
     </row>
@@ -491,13 +491,13 @@
       <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="B7">
+      <c r="B7" t="n">
         <v>2020</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="n">
         <v>17.253</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>3055.83</v>
       </c>
     </row>
@@ -505,13 +505,13 @@
       <c r="A8" t="s">
         <v>6</v>
       </c>
-      <c r="B8">
+      <c r="B8" t="n">
         <v>2020</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="n">
         <v>9.56613</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>1424.4</v>
       </c>
     </row>
@@ -519,13 +519,13 @@
       <c r="A9" t="s">
         <v>7</v>
       </c>
-      <c r="B9">
+      <c r="B9" t="n">
         <v>2020</v>
       </c>
-      <c r="C9">
+      <c r="C9" t="n">
         <v>27.98</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="n">
         <v>3653.91</v>
       </c>
     </row>

</xml_diff>